<commit_message>
Trace where Baseplan's fencing numbers come from and what is missing
Contract 9990776's fence lines are one Pending block for 19-26 Oct, the
same in Baseplan (4), (5), (6) and (7). No docket date and no programme
week gives them. The export's Delivery Dockets sheet is Coates' truck
dockets; its one 9990776 row is the WB13 water barrier delivery.

Baseplan is $96,044.13 short of the 167 signed dockets ($405,150.96
against $309,106.83). It is short $109,528 on fence, scrim, demarcation,
labour, flat feet and blocks, and over $13,484 on relocation, CCB and
ped gates. The demob forecast adds $26,522.40.

Fixed the Fencing sheet's Baseplan total, which priced the 110 m with
hoarding at $16.16 instead of its $23.59: $309,106.83, not
$308,289.53. The fix list and branch tie-out are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Baseplan7_vs_Site_25Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Baseplan7_vs_Site_25Oct2026.xlsx
@@ -41534,7 +41534,7 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>Fence, no scrim (m)</t>
+          <t>Fence, no scrim (m): line 3 at $16.16 + hoarding line 5 at $23.59</t>
         </is>
       </c>
       <c r="B2" s="6" t="n">
@@ -41558,7 +41558,7 @@
         <v>16.16</v>
       </c>
       <c r="H2" s="6" t="n">
-        <v>143630.08</v>
+        <v>144447.38</v>
       </c>
     </row>
     <row r="3">
@@ -41808,7 +41808,7 @@
       <c r="F11" s="6" t="n"/>
       <c r="G11" s="6" t="n"/>
       <c r="H11" s="6" t="n">
-        <v>308289.53</v>
+        <v>309106.83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Check our record against Coates' own delivery dockets
Andrew asked what else needs fixing so our record is right on when
things turned up. arrivals_check.py compares every arrival day and
asset number on the record with the 258 Coates delivery docket rows in
Baseplan (7), and the workbook gains an Arrivals vs dockets sheet.

Most of it agrees: 38 references match their docket's day, 51 dockets
were closed after our day, 13 of 14 barrier dockets and 22 VMS boards
line up. To correct on our record: WC07 1317743 to 1317643, P66 and
P33 fridge numbers, P05's boiling-water unit label. To confirm: GN20
(docket 26102821 out 30 Sep against "never came"), FL01/FL02,
EQ0001-3, EQ0005, WB03, VMS13, VMS09 and T0085/T0109.

The review's GN20 line and its labour move from Remove to Ask Andrew,
and the WC07 number fix now points at our record, not the line.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Baseplan7_vs_Site_25Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Baseplan7_vs_Site_25Oct2026.xlsx
@@ -14,11 +14,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charge lines" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event labour" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fencing (9990776)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generators" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="On site, no line" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch tie-out" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start dates" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since 22 Oct" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arrivals vs dockets" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generators" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="On site, no line" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch tie-out" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start dates" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since 22 Oct" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2641,42 +2642,42 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>9961976</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>52</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Labour Charge: 2 x $333.12</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>1 on site (GN23); GN20 never came</t>
-        </is>
-      </c>
-      <c r="F56" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>1 on site (GN23); the second is GN20, which Andrew said never came (docket 26102821 says 30 Sep)</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
         <is>
           <t>Quantity 1</t>
         </is>
       </c>
-      <c r="G56" s="3" t="n">
+      <c r="G56" s="2" t="n">
         <v>-333.12</v>
       </c>
-      <c r="H56" s="3" t="inlineStr">
-        <is>
-          <t>Baseplan</t>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>Ask Andrew</t>
         </is>
       </c>
     </row>
@@ -3231,42 +3232,42 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="3" t="inlineStr">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>9961976</t>
         </is>
       </c>
-      <c r="B71" s="3" t="inlineStr">
+      <c r="B71" s="2" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C71" s="3" t="inlineStr">
+      <c r="C71" s="2" t="inlineStr">
         <is>
           <t>Remove</t>
         </is>
       </c>
-      <c r="D71" s="3" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>GN20-S01-Generator 365kVA Diesel (1276701) Delivered at $6,260.40</t>
         </is>
       </c>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>GN20's 365 kVA never came (Andrew, 22 Oct 2026: GN20 off the list; record_22Oct2026_gn20_never_came)</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="inlineStr">
-        <is>
-          <t>Close the line (no charge)</t>
-        </is>
-      </c>
-      <c r="G71" s="3" t="n">
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>GN20's 365 kVA: Andrew, 22 Oct 2026, "never came to site 1276701" (record_22Oct2026_gn20_never_came). But Coates' docket 26102821 has it out on 30 Sep, the line is Delivered on that docket, and our record holds a photo filed under GN20/1276701 at 14:14 that day: settle with Andrew before the branch closes the line</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>Close the line (no charge) if it never came; if it came, an In docket and standby to the day it left</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="n">
         <v>-6260.4</v>
       </c>
-      <c r="H71" s="3" t="inlineStr">
-        <is>
-          <t>Baseplan</t>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>Ask Andrew</t>
         </is>
       </c>
     </row>
@@ -3311,40 +3312,40 @@
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="5" t="inlineStr">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>9968955</t>
         </is>
       </c>
-      <c r="B73" s="5" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
         <is>
           <t>38</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr">
+      <c r="C73" s="4" t="inlineStr">
         <is>
           <t>Asset number</t>
         </is>
       </c>
-      <c r="D73" s="5" t="inlineStr">
+      <c r="D73" s="4" t="inlineStr">
         <is>
           <t>WC07 asset 1317643</t>
         </is>
       </c>
-      <c r="E73" s="5" t="inlineStr">
-        <is>
-          <t>WC07 on site carries 1002538, 1002566, 1002651, 1002715, 1083300, 1181004, 1192643, 1200595, 1211959, 1212552, 1317626, 1317632, 1317640, 1317641, 1317647, 1317648, 1317649, 1317652, 1317658, 1317743</t>
-        </is>
-      </c>
-      <c r="F73" s="5" t="inlineStr">
-        <is>
-          <t>Correct the number on the line (the site number stands)</t>
-        </is>
-      </c>
-      <c r="G73" s="5" t="n"/>
-      <c r="H73" s="5" t="inlineStr">
-        <is>
-          <t>Baseplan</t>
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>our record has 1317743; Coates docket 26081411 has 1317643, the same as this line</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
+        <is>
+          <t>Check the unit: our 1317743 is probably a keying slip for 1317643 (correct our record, not the line)</t>
+        </is>
+      </c>
+      <c r="G73" s="4" t="n"/>
+      <c r="H73" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
         </is>
       </c>
     </row>
@@ -3898,6 +3899,162 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Asset no</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Turned up</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>P&amp;L branch</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Building 6m</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>142514</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>KINP</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>HRP</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Building 6m</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>1189410</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>KINP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>FR01</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Fridge</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>1129733</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>KINP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>FR02</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Fridge</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>1157786</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>KINP</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3983,14 +4140,14 @@
         <v>85964.00999999999</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>-3175.12</v>
+        <v>3418.4</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>28071.82</v>
+        <v>21478.3</v>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Ask Andrew · Quantity: $-600.00; Baseplan · Hours: $15.01; Baseplan · Quantity: $-333.12; Baseplan · Rate: $3,403.39; Baseplan · Remove: $-6,260.40; Decision · Rate: $28,671.82</t>
+          <t>Ask Andrew · Quantity: $-933.12; Ask Andrew · Remove: $-6,260.40; Baseplan · Hours: $15.01; Baseplan · Rate: $3,403.39; Decision · Rate: $28,671.82</t>
         </is>
       </c>
     </row>
@@ -4051,10 +4208,10 @@
         <v>1022962.43</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>127387.19</v>
+        <v>133980.71</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>19473.42</v>
+        <v>12879.9</v>
       </c>
       <c r="F6" s="6" t="inlineStr"/>
     </row>
@@ -4063,7 +4220,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10247,7 +10404,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -28385,7 +28542,7 @@
       <c r="N241" s="2" t="n"/>
       <c r="O241" s="2" t="inlineStr">
         <is>
-          <t>GN20's 365 kVA never came (Andrew, 22 Oct 2026: GN20 off the list; record_22Oct2026_gn20_never_came)</t>
+          <t>GN20's 365 kVA: Andrew, 22 Oct 2026, "never came to site 1276701" (record_22Oct2026_gn20_never_came). But Coates' docket 26102821 has it out on 30 Sep, the line is Delivered on that docket, and our record holds a photo filed under GN20/1276701 at 14:14 that day: settle with Andrew before the branch closes the line</t>
         </is>
       </c>
     </row>
@@ -40870,7 +41027,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>1 large set on site: GN23 (GN20 never came)</t>
+          <t>1 large set on site: GN23 (GN20: Andrew said never came; docket 26102821 says 30 Sep)</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -41822,6 +41979,2274 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="70" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Our reference</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Coates docket</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Docket date</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Ours (turned up)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Days ours later</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Finding</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Changes a charge?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>T0002</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>26056582</v>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>1264929</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>LT01 MOLENDINAR Lighting Tower LED Metro</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="5" t="inlineStr">
+        <is>
+          <t>name only: the towers sit on T0002 on our record (Molendinar council yard, 11 Sep)</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>T0002</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>26056582</v>
+      </c>
+      <c r="D3" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>1314284</t>
+        </is>
+      </c>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>LT02 MOLENDINAR Lighting Tower LED Metro</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="inlineStr">
+        <is>
+          <t>name only: as LT01</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>T0002</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>26056582</v>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>1264899</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>LT03 MOLENDINAR Lighting Tower LED 76500lm Hybrid</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n"/>
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>name only: as LT01</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>T0002</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>26056623</v>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>1188888</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>LT04 MOLENDINAR Lighting Tower LED Metro</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n"/>
+      <c r="H5" s="5" t="n"/>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>name only: as LT01</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K5" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>GN20</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>26102821</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>1276701</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>GN20-S01-Generator 365kVA Diesel</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="n"/>
+      <c r="H6" s="2" t="n"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>not on our record</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>GN?</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>26121298</v>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>1316182</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>GN26 CONCERT Generator - 200kVA (Diesel)</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n"/>
+      <c r="H7" s="5" t="n"/>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>name only: the concert sets sit under their own references on our record</t>
+        </is>
+      </c>
+      <c r="J7" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K7" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>GN?</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>26121310</v>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>1316183</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>GN27 CONCERT-Generator - 200kVA (Diesel)</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
+      <c r="H8" s="5" t="n"/>
+      <c r="I8" s="5" t="inlineStr">
+        <is>
+          <t>name only: as GN26</t>
+        </is>
+      </c>
+      <c r="J8" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K8" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>LT06</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>26139060</v>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>1224791</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>LT05/06-Lighting Tower POD Metro</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>name only: the tower pod sits under another reference on our record</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K9" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>26064095</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>1320150</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>P05 Microwave Oven</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>not on our record</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>P05</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>26064095</v>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>1127574</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>P05 Auto Boil</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>our record calls it Aircon; the docket says boiler</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>CP1</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>26064099</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>1116687</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>CP1 Refrigerator - Large</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n"/>
+      <c r="H12" s="2" t="n"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>not on our record</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>CP1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>26064099</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>119810</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>CP1 Urn</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="n"/>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>not on our record</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>P33</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="n">
+        <v>26064103</v>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>1328952</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>P33 Refrigerator - Large</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="n"/>
+      <c r="H14" s="4" t="n"/>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>keying slip: our record has 1238952 on P33</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>P09</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>26076665</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>1254390</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>P09 Auto Boil</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>not on our record</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>HRP</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>26085104</v>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>1189410</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>P36 Portable Building Shell 6.0M x 3.0M - Cyclonic Rated</t>
+        </is>
+      </c>
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="5" t="inlineStr">
+        <is>
+          <t>name only: our record has this shell as HRP (22 Oct review: line 93 is HRP, not P36)</t>
+        </is>
+      </c>
+      <c r="J16" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K16" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>P58</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>26088630</v>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>1273656</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>P44 Portable Building Shell 6.0M x 3.0M - Cyclonic Rated</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="n"/>
+      <c r="H17" s="5" t="n"/>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>name only: our record has this shell as P58 (22 Oct review: line 59 is P58, not P44)</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>P39</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>26094129</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>1272737</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>P38 Refrigerator - Large</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="n"/>
+      <c r="H18" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>on our record under another reference</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>P38</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>26094136</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>1272755</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>P39 Refrigerator - Large</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="n"/>
+      <c r="H19" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>on our record under another reference</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>P66</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="n">
+        <v>26126001</v>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>1311990</t>
+        </is>
+      </c>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>P66 Refrigerator - Large</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="n"/>
+      <c r="H20" s="4" t="n"/>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>keying slip: our record has 131190 on P66</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>P51</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>26126190</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>1328959</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>P46 Refrigerator - Large</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>on our record under another reference</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>P46, P54</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>26126190</v>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>1328957</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>P51 Refrigerator - Large</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>on our record under another reference</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>WC21</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>26064136</v>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>1083399</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>WC21 Toilet Portable - Fresh Water Flush</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>not on our record</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>WC07</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="n">
+        <v>26081411</v>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>1317643</t>
+        </is>
+      </c>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>WC07 Toilet Portable - Fresh Water Flush</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="n"/>
+      <c r="H24" s="4" t="n"/>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>keying slip: our record has 1317743 on WC07</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>WC67</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>26107560</v>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>172824</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>WC01 Toilet Portable - Fresh Water Flush</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="n"/>
+      <c r="H25" s="5" t="n"/>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>placed at WC67 on our record; the docket names WC01 (where it was meant to go)</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Number</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="n">
+        <v>26135873</v>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>1065384</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Laserplane</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>not on our record</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Number on two references</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>P26, P46</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="inlineStr">
+        <is>
+          <t>1311992</t>
+        </is>
+      </c>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>Fridge / Fridge Lge / Furniture</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>one number, two references on our record: keep the one it is on</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Number on two references</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>P28, P46</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>1283996</t>
+        </is>
+      </c>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>Fridge / Fridge Lge / Furniture</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="n"/>
+      <c r="H28" s="4" t="n"/>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>one number, two references on our record: keep the one it is on</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Number on two references</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>FL02, T0004</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="n"/>
+      <c r="D29" s="4" t="n"/>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>1197839</t>
+        </is>
+      </c>
+      <c r="F29" s="4" t="inlineStr">
+        <is>
+          <t>Access &amp; plant / Forklift 2.5T / Other</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="n"/>
+      <c r="H29" s="4" t="n"/>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>one number, two references on our record: keep the one it is on</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>Number on two references</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>T0001, T0103</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="n"/>
+      <c r="D30" s="4" t="n"/>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>1211404</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>VMS / vms5</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="n"/>
+      <c r="H30" s="4" t="n"/>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>one number, two references on our record: keep the one it is on</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Number on two references</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>P41, P62</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="n"/>
+      <c r="D31" s="4" t="n"/>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>1189908</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>Air conditioner</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="n"/>
+      <c r="H31" s="4" t="n"/>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>one number, two references on our record: keep the one it is on</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Number on two references</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>P46, P54</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="n"/>
+      <c r="D32" s="4" t="n"/>
+      <c r="E32" s="4" t="inlineStr">
+        <is>
+          <t>1328957</t>
+        </is>
+      </c>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>Fridge</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="n"/>
+      <c r="H32" s="4" t="n"/>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>one number, two references on our record: keep the one it is on</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>T0002</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>26056582</v>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>1264899</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Lighting towers</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="n"/>
+      <c r="H33" s="5" t="n"/>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>known: the towers went to the Molendinar council yard on 11 Sep, not to site (15 Oct review)</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>no (charged over the event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>T0004</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>26056701</v>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>1197839</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Access &amp; plant</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="n"/>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>no arrival on our record</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>T0243</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="n">
+        <v>26091446</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>1311144</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Toilets &amp; amenities</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="n"/>
+      <c r="H35" s="2" t="n"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>no arrival on our record</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>no (charged over the event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>FL02</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="n">
+        <v>26056701</v>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>1197839</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>docket 14 day(s) before ours</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>EQ0005</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="n">
+        <v>26122181</v>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>1262224</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Access &amp; plant</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>docket 10 day(s) before ours</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>WC06</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="n">
+        <v>26064136</v>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>1195658</t>
+        </is>
+      </c>
+      <c r="F38" s="4" t="inlineStr">
+        <is>
+          <t>Toilets &amp; amenities</t>
+        </is>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>docket 8 day(s) before ours</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>no (charged over the event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>EQ0001</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="n">
+        <v>26133817</v>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>1220903</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>Access &amp; plant</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>docket 3 day(s) before ours</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>T0024</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>26064235</v>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>1211968</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Toilets &amp; amenities</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="inlineStr">
+        <is>
+          <t>2026-09-26</t>
+        </is>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I40" s="5" t="inlineStr">
+        <is>
+          <t>a team reference on its own hire schedule (held out of every charge)</t>
+        </is>
+      </c>
+      <c r="J40" s="5" t="inlineStr">
+        <is>
+          <t>nobody</t>
+        </is>
+      </c>
+      <c r="K40" s="5" t="inlineStr">
+        <is>
+          <t>no (charged over the event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>EQ0002</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="n">
+        <v>26141428</v>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>1300290</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Access &amp; plant</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>docket 1 day(s) before ours</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>EQ0003</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="n">
+        <v>26141448</v>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>1286482</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>Access &amp; plant</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>docket 1 day(s) before ours</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>P44</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="n">
+        <v>26088639</v>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>198481</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="inlineStr">
+        <is>
+          <t>Portable buildings</t>
+        </is>
+      </c>
+      <c r="G43" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H43" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>docket 1 day(s) before ours</t>
+        </is>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>no (charged over the event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>Arrival</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>WC67</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="n">
+        <v>26107560</v>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>172824</t>
+        </is>
+      </c>
+      <c r="F44" s="4" t="inlineStr">
+        <is>
+          <t>Toilets &amp; amenities</t>
+        </is>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="H44" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I44" s="4" t="inlineStr">
+        <is>
+          <t>docket 1 day(s) before ours</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>no (charged over the event)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>Barrier arrival</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>no barrier reference went in that day</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="n">
+        <v>26079322</v>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>ARMORZONMASHTL2</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>WB03 Barrier - Crash Rated Water filled - Armorzone MASH TL2</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="n"/>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>a barrier docket with no matching day on our record (WB03 went in 23 Sep on ours; Baseplan has 18 Sep)</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>VMS arrival</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>VMS09</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="n"/>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>1211404</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>Variable message board</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>docket out 2026-09-07, 2026-10-12; in 2026-10-12</t>
+        </is>
+      </c>
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>VMS arrival</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>VMS13</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="n"/>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>1191957</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>Variable message board</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>docket out 2026-10-16</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -42653,160 +45078,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Asset no</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Turned up</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>P&amp;L branch</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Building 6m</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>142514</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>KINP</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>HRP</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Building 6m</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>1189410</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>KINP</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>FR01</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Fridge</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>1129733</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>KINP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>FR02</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Fridge</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>1157786</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>KINP</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Settle GN20 1276701: never came to site
Andrew confirmed again that the 365 kVA set 1276701 never came to
site. The review puts 9961976 line 6 and the second large-set labour
line back to Remove for the branch, which reverses Coates' docket
26102821 and the line's Delivered status. NVAC fixes are back to
-$3,175.12.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Baseplan7_vs_Site_25Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Baseplan7_vs_Site_25Oct2026.xlsx
@@ -2642,42 +2642,42 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>9961976</t>
         </is>
       </c>
-      <c r="B56" s="2" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>52</t>
         </is>
       </c>
-      <c r="C56" s="2" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D56" s="2" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>Labour Charge: 2 x $333.12</t>
         </is>
       </c>
-      <c r="E56" s="2" t="inlineStr">
-        <is>
-          <t>1 on site (GN23); the second is GN20, which Andrew said never came (docket 26102821 says 30 Sep)</t>
-        </is>
-      </c>
-      <c r="F56" s="2" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>1 on site (GN23); the second was GN20, which never came to site (Andrew, 22 and 25 Oct)</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
         <is>
           <t>Quantity 1</t>
         </is>
       </c>
-      <c r="G56" s="2" t="n">
+      <c r="G56" s="3" t="n">
         <v>-333.12</v>
       </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>Ask Andrew</t>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>Baseplan</t>
         </is>
       </c>
     </row>
@@ -3232,42 +3232,42 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="inlineStr">
+      <c r="A71" s="3" t="inlineStr">
         <is>
           <t>9961976</t>
         </is>
       </c>
-      <c r="B71" s="2" t="inlineStr">
+      <c r="B71" s="3" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="C71" s="2" t="inlineStr">
+      <c r="C71" s="3" t="inlineStr">
         <is>
           <t>Remove</t>
         </is>
       </c>
-      <c r="D71" s="2" t="inlineStr">
+      <c r="D71" s="3" t="inlineStr">
         <is>
           <t>GN20-S01-Generator 365kVA Diesel (1276701) Delivered at $6,260.40</t>
         </is>
       </c>
-      <c r="E71" s="2" t="inlineStr">
-        <is>
-          <t>GN20's 365 kVA: Andrew, 22 Oct 2026, "never came to site 1276701" (record_22Oct2026_gn20_never_came). But Coates' docket 26102821 has it out on 30 Sep, the line is Delivered on that docket, and our record holds a photo filed under GN20/1276701 at 14:14 that day: settle with Andrew before the branch closes the line</t>
-        </is>
-      </c>
-      <c r="F71" s="2" t="inlineStr">
-        <is>
-          <t>Close the line (no charge) if it never came; if it came, an In docket and standby to the day it left</t>
-        </is>
-      </c>
-      <c r="G71" s="2" t="n">
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>GN20's 365 kVA never came to site (Andrew, 22 Oct 2026, and again 25 Oct: "this never came to site 1276701 Generator 365kVA Diesel"). Coates' docket 26102821 (out 30 Sep) and the line's Delivered status are wrong: the branch reverses the docket</t>
+        </is>
+      </c>
+      <c r="F71" s="3" t="inlineStr">
+        <is>
+          <t>Reverse docket 26102821 and close the line (no charge)</t>
+        </is>
+      </c>
+      <c r="G71" s="3" t="n">
         <v>-6260.4</v>
       </c>
-      <c r="H71" s="2" t="inlineStr">
-        <is>
-          <t>Ask Andrew</t>
+      <c r="H71" s="3" t="inlineStr">
+        <is>
+          <t>Baseplan</t>
         </is>
       </c>
     </row>
@@ -4140,14 +4140,14 @@
         <v>85964.00999999999</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>3418.4</v>
+        <v>-3175.12</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>21478.3</v>
+        <v>28071.82</v>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Ask Andrew · Quantity: $-933.12; Ask Andrew · Remove: $-6,260.40; Baseplan · Hours: $15.01; Baseplan · Rate: $3,403.39; Decision · Rate: $28,671.82</t>
+          <t>Ask Andrew · Quantity: $-600.00; Baseplan · Hours: $15.01; Baseplan · Quantity: $-333.12; Baseplan · Rate: $3,403.39; Baseplan · Remove: $-6,260.40; Decision · Rate: $28,671.82</t>
         </is>
       </c>
     </row>
@@ -4208,10 +4208,10 @@
         <v>1022962.43</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>133980.71</v>
+        <v>127387.19</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>12879.9</v>
+        <v>19473.42</v>
       </c>
       <c r="F6" s="6" t="inlineStr"/>
     </row>
@@ -28542,7 +28542,7 @@
       <c r="N241" s="2" t="n"/>
       <c r="O241" s="2" t="inlineStr">
         <is>
-          <t>GN20's 365 kVA: Andrew, 22 Oct 2026, "never came to site 1276701" (record_22Oct2026_gn20_never_came). But Coates' docket 26102821 has it out on 30 Sep, the line is Delivered on that docket, and our record holds a photo filed under GN20/1276701 at 14:14 that day: settle with Andrew before the branch closes the line</t>
+          <t>GN20's 365 kVA never came to site (Andrew, 22 Oct 2026, and again 25 Oct: "this never came to site 1276701 Generator 365kVA Diesel"). Coates' docket 26102821 (out 30 Sep) and the line's Delivered status are wrong: the branch reverses the docket</t>
         </is>
       </c>
     </row>
@@ -41027,7 +41027,7 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>1 large set on site: GN23 (GN20: Andrew said never came; docket 26102821 says 30 Sep)</t>
+          <t>1 large set on site: GN23 (GN20 never came to site; Andrew, 22 and 25 Oct)</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -42241,47 +42241,47 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Number</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>GN20</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
+      <c r="C6" s="4" t="n">
         <v>26102821</v>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>2026-09-30</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" s="4" t="inlineStr">
         <is>
           <t>1276701</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" s="4" t="inlineStr">
         <is>
           <t>GN20-S01-Generator 365kVA Diesel</t>
         </is>
       </c>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>not on our record</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="G6" s="4" t="n"/>
+      <c r="H6" s="4" t="n"/>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>never came to site (Andrew, 22 and 25 Oct): the docket is wrong; the branch reverses it and closes line 6</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Baseplan</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
         <is>
           <t>no</t>
         </is>

</xml_diff>

<commit_message>
Add the four building items and the laserplane to the record
Andrew confirmed they are on site and asked for them to be added.
Through the page's own controls, record 10824 to 10847, verified:
Microwave 1320150 on P05, Fridge 1116687 and Urn 119810 on CP1 (each
onto the schedule's unnumbered row), Zip boiler 1254390 on P09, and
EQ0006 Laserplane 1065384 under Other with its contract line note,
MEAD, quantity 1, on site and complete. Today's Equipment stays 12/12
and the P&L by branch is unchanged. The backup stays private.

The Baseplan (7) review follows Andrew's ruling that our record is
the truth and only Baseplan matters: the docket cross-check sheet is
out of the workbook, WC07's line takes our number, and generator
transport agrees at 10 legs with GN10's swap on our record.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Baseplan7_vs_Site_25Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Baseplan7_vs_Site_25Oct2026.xlsx
@@ -14,12 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charge lines" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Event labour" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fencing (9990776)" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arrivals vs dockets" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generators" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="On site, no line" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch tie-out" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start dates" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since 22 Oct" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generators" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="On site, no line" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Branch tie-out" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start dates" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Since 22 Oct" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -466,7 +465,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H87"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2682,54 +2681,52 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>9961976</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>53</t>
-        </is>
-      </c>
-      <c r="C57" s="2" t="inlineStr">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
+          <t>9968955</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>84, 140</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D57" s="2" t="inlineStr">
-        <is>
-          <t>Transport Charge: 10 x $300.00</t>
-        </is>
-      </c>
-      <c r="E57" s="2" t="inlineStr">
-        <is>
-          <t>8 on site (GN03, GN04, GN10, GN25)</t>
-        </is>
-      </c>
-      <c r="F57" s="2" t="inlineStr">
-        <is>
-          <t>Quantity 8</t>
-        </is>
-      </c>
-      <c r="G57" s="2" t="n">
-        <v>-600</v>
-      </c>
-      <c r="H57" s="2" t="inlineStr">
-        <is>
-          <t>Ask Andrew</t>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>WC67 FWF: 3 on hire</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>WC67 has 4 FWF on site (arrived Thu 01 Oct)</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Add 1 FWF (hire line)</t>
+        </is>
+      </c>
+      <c r="G57" s="3" t="n"/>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>Baseplan</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>9968955</t>
+          <t>9972648/9990776</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>84, 140</t>
+          <t>-</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -2739,17 +2736,17 @@
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>WC67 FWF: 3 on hire</t>
+          <t>WB07: 0 barriers</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>WC67 has 4 FWF on site (arrived Thu 01 Oct)</t>
+          <t>WB07: 17 on site</t>
         </is>
       </c>
       <c r="F58" s="3" t="inlineStr">
         <is>
-          <t>Add 1 FWF (hire line)</t>
+          <t>Match the quantity to the site count (barriers are charged from when they go in)</t>
         </is>
       </c>
       <c r="G58" s="3" t="n"/>
@@ -2767,7 +2764,7 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -2777,12 +2774,12 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>WB07: 0 barriers</t>
+          <t>WB05: 12 barriers</t>
         </is>
       </c>
       <c r="E59" s="3" t="inlineStr">
         <is>
-          <t>WB07: 17 on site</t>
+          <t>WB05: 13 on site</t>
         </is>
       </c>
       <c r="F59" s="3" t="inlineStr">
@@ -2805,7 +2802,7 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -2815,12 +2812,12 @@
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>WB05: 12 barriers</t>
+          <t>WB04: 13 barriers</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>WB05: 13 on site</t>
+          <t>WB04: 14 on site</t>
         </is>
       </c>
       <c r="F60" s="3" t="inlineStr">
@@ -2838,12 +2835,12 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>9972648/9990776</t>
+          <t>9990776</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
@@ -2853,20 +2850,22 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>WB04: 13 barriers</t>
+          <t>Ped Gates: 32</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
         <is>
-          <t>WB04: 14 on site</t>
+          <t>22 on the signed dockets (to 25 Oct)</t>
         </is>
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>Match the quantity to the site count (barriers are charged from when they go in)</t>
-        </is>
-      </c>
-      <c r="G61" s="3" t="n"/>
+          <t>Quantity 22</t>
+        </is>
+      </c>
+      <c r="G61" s="3" t="n">
+        <v>-361.8</v>
+      </c>
       <c r="H61" s="3" t="inlineStr">
         <is>
           <t>Baseplan</t>
@@ -2881,7 +2880,7 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3, 5</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -2891,21 +2890,21 @@
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Ped Gates: 32</t>
+          <t>1.8 m security fence 8778 m + with hoarding 110 m</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>22 on the signed dockets (to 25 Oct)</t>
+          <t>13270 m of fence with no scrim on the signed dockets</t>
         </is>
       </c>
       <c r="F62" s="3" t="inlineStr">
         <is>
-          <t>Quantity 22</t>
+          <t>Quantity 13160 m on line 3 (keep the 110 m with hoarding on line 5 if it is in the dockets' clean metres)</t>
         </is>
       </c>
       <c r="G62" s="3" t="n">
-        <v>-361.8</v>
+        <v>70813.12</v>
       </c>
       <c r="H62" s="3" t="inlineStr">
         <is>
@@ -2921,7 +2920,7 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>3, 5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2931,21 +2930,21 @@
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>1.8 m security fence 8778 m + with hoarding 110 m</t>
+          <t>Fence Relocation: 1520</t>
         </is>
       </c>
       <c r="E63" s="3" t="inlineStr">
         <is>
-          <t>13270 m of fence with no scrim on the signed dockets</t>
+          <t>137.5 on the signed dockets (to 25 Oct); demob relocation still to come</t>
         </is>
       </c>
       <c r="F63" s="3" t="inlineStr">
         <is>
-          <t>Quantity 13160 m on line 3 (keep the 110 m with hoarding on line 5 if it is in the dockets' clean metres)</t>
+          <t>Quantity 137.5 to date</t>
         </is>
       </c>
       <c r="G63" s="3" t="n">
-        <v>70813.12</v>
+        <v>-11958.62</v>
       </c>
       <c r="H63" s="3" t="inlineStr">
         <is>
@@ -2961,7 +2960,7 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -2971,21 +2970,21 @@
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>Fence Relocation: 1520</t>
+          <t>1.8m Fence w/Scrim: 2775</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>137.5 on the signed dockets (to 25 Oct); demob relocation still to come</t>
+          <t>3977.5 m of fence with scrim on the signed dockets (to 25 Oct)</t>
         </is>
       </c>
       <c r="F64" s="3" t="inlineStr">
         <is>
-          <t>Quantity 137.5 to date</t>
+          <t>Quantity 3977.5</t>
         </is>
       </c>
       <c r="G64" s="3" t="n">
-        <v>-11958.62</v>
+        <v>19432.4</v>
       </c>
       <c r="H64" s="3" t="inlineStr">
         <is>
@@ -3001,7 +3000,7 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -3011,21 +3010,21 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>1.8m Fence w/Scrim: 2775</t>
+          <t>Barrier - Crowd Control: 2350</t>
         </is>
       </c>
       <c r="E65" s="3" t="inlineStr">
         <is>
-          <t>3977.5 m of fence with scrim on the signed dockets (to 25 Oct)</t>
+          <t>2195 on the signed dockets (to 25 Oct)</t>
         </is>
       </c>
       <c r="F65" s="3" t="inlineStr">
         <is>
-          <t>Quantity 3977.5</t>
+          <t>Quantity 2195</t>
         </is>
       </c>
       <c r="G65" s="3" t="n">
-        <v>19432.4</v>
+        <v>-1164.05</v>
       </c>
       <c r="H65" s="3" t="inlineStr">
         <is>
@@ -3041,7 +3040,7 @@
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -3051,21 +3050,21 @@
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Barrier - Crowd Control: 2350</t>
+          <t>Barrier - Crowd Control Flat Feet: 220</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>2195 on the signed dockets (to 25 Oct)</t>
+          <t>270 on the signed dockets (to 25 Oct)</t>
         </is>
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>Quantity 2195</t>
+          <t>Quantity 270</t>
         </is>
       </c>
       <c r="G66" s="3" t="n">
-        <v>-1164.05</v>
+        <v>375.5</v>
       </c>
       <c r="H66" s="3" t="inlineStr">
         <is>
@@ -3081,7 +3080,7 @@
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -3091,21 +3090,21 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>Barrier - Crowd Control Flat Feet: 220</t>
+          <t>Demarcation CCB: 4603</t>
         </is>
       </c>
       <c r="E67" s="3" t="inlineStr">
         <is>
-          <t>270 on the signed dockets (to 25 Oct)</t>
+          <t>5062.5 on the signed dockets (to 25 Oct)</t>
         </is>
       </c>
       <c r="F67" s="3" t="inlineStr">
         <is>
-          <t>Quantity 270</t>
+          <t>Quantity 5062.5</t>
         </is>
       </c>
       <c r="G67" s="3" t="n">
-        <v>375.5</v>
+        <v>6010.26</v>
       </c>
       <c r="H67" s="3" t="inlineStr">
         <is>
@@ -3121,7 +3120,7 @@
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -3131,21 +3130,21 @@
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>Demarcation CCB: 4603</t>
+          <t>Shade Cloth: 2775</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>5062.5 on the signed dockets (to 25 Oct)</t>
+          <t>3977.5 m of fence with scrim on the signed dockets (to 25 Oct)</t>
         </is>
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>Quantity 5062.5</t>
+          <t>Quantity 3977.5</t>
         </is>
       </c>
       <c r="G68" s="3" t="n">
-        <v>6010.26</v>
+        <v>11267.43</v>
       </c>
       <c r="H68" s="3" t="inlineStr">
         <is>
@@ -3154,92 +3153,92 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="inlineStr">
-        <is>
-          <t>9990776</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="C69" s="3" t="inlineStr">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>our P&amp;L</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>servicing</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>Shade Cloth: 2775</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>3977.5 m of fence with scrim on the signed dockets (to 25 Oct)</t>
-        </is>
-      </c>
-      <c r="F69" s="3" t="inlineStr">
-        <is>
-          <t>Quantity 3977.5</t>
-        </is>
-      </c>
-      <c r="G69" s="3" t="n">
-        <v>11267.43</v>
-      </c>
-      <c r="H69" s="3" t="inlineStr">
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>the P&amp;L charges WC31's two 16-pan blocks as sewer-connect cleans (2 x 3 x $260.25 = $1,561.50)</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>they are pumped out every night (servicing tracker), as Baseplan line 142 charges them (2 x 3 x $624.60 = $3,747.60)</t>
+        </is>
+      </c>
+      <c r="F69" s="4" t="inlineStr">
+        <is>
+          <t>Count the 16-pans with the tank pump-outs on Costs (P&amp;L +$2,186.10)</t>
+        </is>
+      </c>
+      <c r="G69" s="4" t="n"/>
+      <c r="H69" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>9961976</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Remove</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>GN20-S01-Generator 365kVA Diesel (1276701) Delivered at $6,260.40</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>GN20's 365 kVA never came to site (Andrew, 22 Oct 2026, and again 25 Oct: "this never came to site 1276701 Generator 365kVA Diesel"). Coates' docket 26102821 (out 30 Sep) and the line's Delivered status are wrong: the branch reverses the docket</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Reverse docket 26102821 and close the line (no charge)</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="n">
+        <v>-6260.4</v>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
         <is>
           <t>Baseplan</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="4" t="inlineStr">
-        <is>
-          <t>our P&amp;L</t>
-        </is>
-      </c>
-      <c r="B70" s="4" t="inlineStr">
-        <is>
-          <t>servicing</t>
-        </is>
-      </c>
-      <c r="C70" s="4" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="D70" s="4" t="inlineStr">
-        <is>
-          <t>the P&amp;L charges WC31's two 16-pan blocks as sewer-connect cleans (2 x 3 x $260.25 = $1,561.50)</t>
-        </is>
-      </c>
-      <c r="E70" s="4" t="inlineStr">
-        <is>
-          <t>they are pumped out every night (servicing tracker), as Baseplan line 142 charges them (2 x 3 x $624.60 = $3,747.60)</t>
-        </is>
-      </c>
-      <c r="F70" s="4" t="inlineStr">
-        <is>
-          <t>Count the 16-pans with the tank pump-outs on Costs (P&amp;L +$2,186.10)</t>
-        </is>
-      </c>
-      <c r="G70" s="4" t="n"/>
-      <c r="H70" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>9961976</t>
+          <t>9968955</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>154</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
@@ -3249,21 +3248,21 @@
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>GN20-S01-Generator 365kVA Diesel (1276701) Delivered at $6,260.40</t>
+          <t>PG29 Toilet FWF at $90.07</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
         <is>
-          <t>GN20's 365 kVA never came to site (Andrew, 22 Oct 2026, and again 25 Oct: "this never came to site 1276701 Generator 365kVA Diesel"). Coates' docket 26102821 (out 30 Sep) and the line's Delivered status are wrong: the branch reverses the docket</t>
+          <t>PG29 is on its own hire schedule (held out of every charge, Andrew 23 Oct)</t>
         </is>
       </c>
       <c r="F71" s="3" t="inlineStr">
         <is>
-          <t>Reverse docket 26102821 and close the line (no charge)</t>
+          <t>Take the line off this contract</t>
         </is>
       </c>
       <c r="G71" s="3" t="n">
-        <v>-6260.4</v>
+        <v>-90.06999999999999</v>
       </c>
       <c r="H71" s="3" t="inlineStr">
         <is>
@@ -3272,80 +3271,80 @@
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
+      <c r="A72" s="5" t="inlineStr">
         <is>
           <t>9968955</t>
         </is>
       </c>
-      <c r="B72" s="3" t="inlineStr">
-        <is>
-          <t>154</t>
-        </is>
-      </c>
-      <c r="C72" s="3" t="inlineStr">
-        <is>
-          <t>Remove</t>
-        </is>
-      </c>
-      <c r="D72" s="3" t="inlineStr">
-        <is>
-          <t>PG29 Toilet FWF at $90.07</t>
-        </is>
-      </c>
-      <c r="E72" s="3" t="inlineStr">
-        <is>
-          <t>PG29 is on its own hire schedule (held out of every charge, Andrew 23 Oct)</t>
-        </is>
-      </c>
-      <c r="F72" s="3" t="inlineStr">
-        <is>
-          <t>Take the line off this contract</t>
-        </is>
-      </c>
-      <c r="G72" s="3" t="n">
-        <v>-90.06999999999999</v>
-      </c>
-      <c r="H72" s="3" t="inlineStr">
+      <c r="B72" s="5" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Asset number</t>
+        </is>
+      </c>
+      <c r="D72" s="5" t="inlineStr">
+        <is>
+          <t>WC07 asset 1317643</t>
+        </is>
+      </c>
+      <c r="E72" s="5" t="inlineStr">
+        <is>
+          <t>WC07 on site carries 1002538, 1002566, 1002651, 1002715, 1083300, 1181004, 1192643, 1200595, 1211959, 1212552, 1317626, 1317632, 1317640, 1317641, 1317647, 1317648, 1317649, 1317652, 1317658, 1317743</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>Correct the number on the line (the site number stands)</t>
+        </is>
+      </c>
+      <c r="G72" s="5" t="n"/>
+      <c r="H72" s="5" t="inlineStr">
         <is>
           <t>Baseplan</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="4" t="inlineStr">
-        <is>
-          <t>9968955</t>
-        </is>
-      </c>
-      <c r="B73" s="4" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="C73" s="4" t="inlineStr">
-        <is>
-          <t>Asset number</t>
-        </is>
-      </c>
-      <c r="D73" s="4" t="inlineStr">
-        <is>
-          <t>WC07 asset 1317643</t>
-        </is>
-      </c>
-      <c r="E73" s="4" t="inlineStr">
-        <is>
-          <t>our record has 1317743; Coates docket 26081411 has 1317643, the same as this line</t>
-        </is>
-      </c>
-      <c r="F73" s="4" t="inlineStr">
-        <is>
-          <t>Check the unit: our 1317743 is probably a keying slip for 1317643 (correct our record, not the line)</t>
-        </is>
-      </c>
-      <c r="G73" s="4" t="n"/>
-      <c r="H73" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
+      <c r="A73" s="5" t="inlineStr">
+        <is>
+          <t>9961265</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>Start date</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>VMS22 445T Variable Message Board Senior Premiair: start Wed 21 Oct</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>on site Thu 22 Oct (Andrew's word (22 Oct) / pin on site)</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>Start Thu 22 Oct (VMS is charged from when it goes in)</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="n">
+        <v>53.61</v>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>Baseplan</t>
         </is>
       </c>
     </row>
@@ -3357,7 +3356,7 @@
       </c>
       <c r="B74" s="5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>31</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
@@ -3367,7 +3366,7 @@
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>VMS22 445T Variable Message Board Senior Premiair: start Wed 21 Oct</t>
+          <t>VMS24 450T Variable Message Board Senior: start Mon 19 Oct</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -3381,7 +3380,7 @@
         </is>
       </c>
       <c r="G74" s="5" t="n">
-        <v>53.61</v>
+        <v>160.83</v>
       </c>
       <c r="H74" s="5" t="inlineStr">
         <is>
@@ -3397,7 +3396,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>34</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
@@ -3407,21 +3406,21 @@
       </c>
       <c r="D75" s="5" t="inlineStr">
         <is>
-          <t>VMS24 450T Variable Message Board Senior: start Mon 19 Oct</t>
+          <t>VMS14 Variable Message Board Junior: start Mon 19 Oct</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>on site Thu 22 Oct (Andrew's word (22 Oct) / pin on site)</t>
+          <t>on site Fri 16 Oct (recorded on site (load T0158))</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>Start Thu 22 Oct (VMS is charged from when it goes in)</t>
+          <t>Start Fri 16 Oct (VMS is charged from when it goes in)</t>
         </is>
       </c>
       <c r="G75" s="5" t="n">
-        <v>160.83</v>
+        <v>-160.83</v>
       </c>
       <c r="H75" s="5" t="inlineStr">
         <is>
@@ -3437,7 +3436,7 @@
       </c>
       <c r="B76" s="5" t="inlineStr">
         <is>
-          <t>34</t>
+          <t>35</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
@@ -3447,7 +3446,7 @@
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>VMS14 Variable Message Board Junior: start Mon 19 Oct</t>
+          <t>VMS15 Variable Message Board Senior: start Mon 19 Oct</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -3477,7 +3476,7 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>35</t>
+          <t>37</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
@@ -3487,7 +3486,7 @@
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>VMS15 Variable Message Board Senior: start Mon 19 Oct</t>
+          <t>VMS16 Variable Message Board Senior: start Mon 19 Oct</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -3517,7 +3516,7 @@
       </c>
       <c r="B78" s="5" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>39</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
@@ -3527,7 +3526,7 @@
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>VMS16 Variable Message Board Senior: start Mon 19 Oct</t>
+          <t>VMS17 Variable Message Board Senior: start Mon 19 Oct</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -3552,12 +3551,12 @@
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
         <is>
-          <t>9961265</t>
+          <t>9961976</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>48</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
@@ -3567,22 +3566,20 @@
       </c>
       <c r="D79" s="5" t="inlineStr">
         <is>
-          <t>VMS17 Variable Message Board Senior: start Mon 19 Oct</t>
+          <t>GN06 Generator - 60kVA (Diesel): start Mon 19 Oct</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
         <is>
-          <t>on site Fri 16 Oct (recorded on site (load T0158))</t>
+          <t>GN06 first on site Thu 15 Oct</t>
         </is>
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Start Fri 16 Oct (VMS is charged from when it goes in)</t>
-        </is>
-      </c>
-      <c r="G79" s="5" t="n">
-        <v>-160.83</v>
-      </c>
+          <t>Start Thu 15 Oct (charged from when it goes in)</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="n"/>
       <c r="H79" s="5" t="inlineStr">
         <is>
           <t>Baseplan</t>
@@ -3592,12 +3589,12 @@
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
         <is>
-          <t>9961976</t>
+          <t>9972648</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -3607,17 +3604,17 @@
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>GN06 Generator - 60kVA (Diesel): start Mon 19 Oct</t>
+          <t>WB03 Barrier - Crash Rated Water filled - Armorzon: start Fri 18 Sep</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
         <is>
-          <t>GN06 first on site Thu 15 Oct</t>
+          <t>WB03 first on site Wed 23 Sep</t>
         </is>
       </c>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Start Thu 15 Oct (charged from when it goes in)</t>
+          <t>Start Wed 23 Sep (charged from when it goes in)</t>
         </is>
       </c>
       <c r="G80" s="5" t="n"/>
@@ -3628,40 +3625,40 @@
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="5" t="inlineStr">
-        <is>
-          <t>9972648</t>
-        </is>
-      </c>
-      <c r="B81" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="C81" s="5" t="inlineStr">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>9987005</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
         <is>
           <t>Start date</t>
         </is>
       </c>
-      <c r="D81" s="5" t="inlineStr">
-        <is>
-          <t>WB03 Barrier - Crash Rated Water filled - Armorzon: start Fri 18 Sep</t>
-        </is>
-      </c>
-      <c r="E81" s="5" t="inlineStr">
-        <is>
-          <t>WB03 first on site Wed 23 Sep</t>
-        </is>
-      </c>
-      <c r="F81" s="5" t="inlineStr">
-        <is>
-          <t>Start Wed 23 Sep (charged from when it goes in)</t>
-        </is>
-      </c>
-      <c r="G81" s="5" t="n"/>
-      <c r="H81" s="5" t="inlineStr">
-        <is>
-          <t>Baseplan</t>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Supply Forklift 5.0t Diesel: start Mon 05 Oct</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>T0085 first on site Mon 28 Sep (machines changed on some plant references: confirm this unit's day)</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>Start Mon 28 Sep (charged from when it goes in)</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="n"/>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>Ask Andrew</t>
         </is>
       </c>
     </row>
@@ -3673,7 +3670,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -3683,17 +3680,17 @@
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>Supply Forklift 5.0t Diesel: start Mon 05 Oct</t>
+          <t>Supply Telehandler Fork Extension 1800mm: start Mon 05 Oct</t>
         </is>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>T0085 first on site Mon 28 Sep (machines changed on some plant references: confirm this unit's day)</t>
+          <t>EQ0005 first on site Fri 23 Oct (machines changed on some plant references: confirm this unit's day)</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>Start Mon 28 Sep (charged from when it goes in)</t>
+          <t>Start Fri 23 Oct (charged from when it goes in)</t>
         </is>
       </c>
       <c r="G82" s="2" t="n"/>
@@ -3711,7 +3708,7 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -3721,17 +3718,17 @@
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
-          <t>Supply Telehandler Fork Extension 1800mm: start Mon 05 Oct</t>
+          <t>Forklift Rough Terrain 2.5t 4WD Diesel: start Tue 13 Oct</t>
         </is>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>EQ0005 first on site Fri 23 Oct (machines changed on some plant references: confirm this unit's day)</t>
+          <t>T0109 first on site Mon 28 Sep (machines changed on some plant references: confirm this unit's day)</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>Start Fri 23 Oct (charged from when it goes in)</t>
+          <t>Start Mon 28 Sep (charged from when it goes in)</t>
         </is>
       </c>
       <c r="G83" s="2" t="n"/>
@@ -3744,12 +3741,12 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>9987005</t>
+          <t>9992300</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -3759,17 +3756,17 @@
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Forklift Rough Terrain 2.5t 4WD Diesel: start Tue 13 Oct</t>
+          <t>Scissor Lift With Operator Protection 43ft (13.0M): start Mon 19 Oct</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>T0109 first on site Mon 28 Sep (machines changed on some plant references: confirm this unit's day)</t>
+          <t>EQ0001 first on site Thu 22 Oct (machines changed on some plant references: confirm this unit's day)</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>Start Mon 28 Sep (charged from when it goes in)</t>
+          <t>Start Thu 22 Oct (charged from when it goes in)</t>
         </is>
       </c>
       <c r="G84" s="2" t="n"/>
@@ -3780,40 +3777,40 @@
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>9992300</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="C85" s="2" t="inlineStr">
+      <c r="A85" s="5" t="inlineStr">
+        <is>
+          <t>9994954</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
         <is>
           <t>Start date</t>
         </is>
       </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>Scissor Lift With Operator Protection 43ft (13.0M): start Mon 19 Oct</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>EQ0001 first on site Thu 22 Oct (machines changed on some plant references: confirm this unit's day)</t>
-        </is>
-      </c>
-      <c r="F85" s="2" t="inlineStr">
-        <is>
-          <t>Start Thu 22 Oct (charged from when it goes in)</t>
-        </is>
-      </c>
-      <c r="G85" s="2" t="n"/>
-      <c r="H85" s="2" t="inlineStr">
-        <is>
-          <t>Ask Andrew</t>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>GN26 Generator - 200kVA (Diesel): start Fri 23 Oct</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>GN? first on site Mon 12 Oct</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Start Mon 12 Oct (charged from when it goes in)</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="n"/>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>Baseplan</t>
         </is>
       </c>
     </row>
@@ -3825,7 +3822,7 @@
       </c>
       <c r="B86" s="5" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>11</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -3835,7 +3832,7 @@
       </c>
       <c r="D86" s="5" t="inlineStr">
         <is>
-          <t>GN26 Generator - 200kVA (Diesel): start Fri 23 Oct</t>
+          <t>GN27 Generator - 200kVA (Diesel): start Fri 23 Oct</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -3850,44 +3847,6 @@
       </c>
       <c r="G86" s="5" t="n"/>
       <c r="H86" s="5" t="inlineStr">
-        <is>
-          <t>Baseplan</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="5" t="inlineStr">
-        <is>
-          <t>9994954</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>Start date</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="inlineStr">
-        <is>
-          <t>GN27 Generator - 200kVA (Diesel): start Fri 23 Oct</t>
-        </is>
-      </c>
-      <c r="E87" s="5" t="inlineStr">
-        <is>
-          <t>GN? first on site Mon 12 Oct</t>
-        </is>
-      </c>
-      <c r="F87" s="5" t="inlineStr">
-        <is>
-          <t>Start Mon 12 Oct (charged from when it goes in)</t>
-        </is>
-      </c>
-      <c r="G87" s="5" t="n"/>
-      <c r="H87" s="5" t="inlineStr">
         <is>
           <t>Baseplan</t>
         </is>
@@ -3899,162 +3858,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Asset no</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Turned up</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>P&amp;L branch</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="6" t="inlineStr">
-        <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>Building 6m</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>142514</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="inlineStr">
-        <is>
-          <t>KINP</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>HRP</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="inlineStr">
-        <is>
-          <t>Building 6m</t>
-        </is>
-      </c>
-      <c r="C3" s="6" t="inlineStr">
-        <is>
-          <t>1189410</t>
-        </is>
-      </c>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="E3" s="6" t="inlineStr">
-        <is>
-          <t>KINP</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>FR01</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Fridge</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>1129733</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>KINP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>FR02</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>Fridge</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>1157786</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>2026-10-17</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>KINP</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4143,11 +3946,11 @@
         <v>-3175.12</v>
       </c>
       <c r="E3" s="6" t="n">
-        <v>28071.82</v>
+        <v>28671.82</v>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Ask Andrew · Quantity: $-600.00; Baseplan · Hours: $15.01; Baseplan · Quantity: $-333.12; Baseplan · Rate: $3,403.39; Baseplan · Remove: $-6,260.40; Decision · Rate: $28,671.82</t>
+          <t>Baseplan · Hours: $15.01; Baseplan · Quantity: $-333.12; Baseplan · Rate: $3,403.39; Baseplan · Remove: $-6,260.40; Decision · Rate: $28,671.82</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4014,7 @@
         <v>127387.19</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>19473.42</v>
+        <v>20073.42</v>
       </c>
       <c r="F6" s="6" t="inlineStr"/>
     </row>
@@ -4220,7 +4023,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10404,7 +10207,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14221,7 +14024,7 @@
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>nothing on the record carries this line</t>
+          <t>EQ0006 on our record since 25 Oct (Andrew: on site; record_25Oct2026_accessories_laserplane)</t>
         </is>
       </c>
     </row>
@@ -41047,52 +40850,52 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>9961976</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B27" s="5" t="inlineStr">
         <is>
           <t>53</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Transport Charge</t>
         </is>
       </c>
-      <c r="D27" s="2" t="n">
+      <c r="D27" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="E27" s="2" t="n">
+      <c r="E27" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="F27" s="2" t="n">
+      <c r="F27" s="5" t="n">
         <v>3000</v>
       </c>
-      <c r="G27" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="H27" s="2" t="n">
-        <v>2400</v>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>4 sets up to 30 kVA (GN03, GN04, GN10, GN25) x 2 legs</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>Baseplan 10, ours 8</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="G27" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>3000</v>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>4 sets up to 30 kVA (GN03, GN04, GN10, GN25) x 2 legs + 2 for each swap on our record (GN10)</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>agrees</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
         <is>
           <t>NVAC-FRI</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="L27" s="5" t="inlineStr">
         <is>
           <t>NVAC</t>
         </is>
@@ -41979,2274 +41782,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K47"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="34" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="70" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Our reference</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Coates docket</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Docket date</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>What</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Ours (turned up)</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Days ours later</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Finding</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Who</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Changes a charge?</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B2" s="5" t="inlineStr">
-        <is>
-          <t>T0002</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="n">
-        <v>26056582</v>
-      </c>
-      <c r="D2" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="E2" s="5" t="inlineStr">
-        <is>
-          <t>1264929</t>
-        </is>
-      </c>
-      <c r="F2" s="5" t="inlineStr">
-        <is>
-          <t>LT01 MOLENDINAR Lighting Tower LED Metro</t>
-        </is>
-      </c>
-      <c r="G2" s="5" t="n"/>
-      <c r="H2" s="5" t="n"/>
-      <c r="I2" s="5" t="inlineStr">
-        <is>
-          <t>name only: the towers sit on T0002 on our record (Molendinar council yard, 11 Sep)</t>
-        </is>
-      </c>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="inlineStr">
-        <is>
-          <t>T0002</t>
-        </is>
-      </c>
-      <c r="C3" s="5" t="n">
-        <v>26056582</v>
-      </c>
-      <c r="D3" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="inlineStr">
-        <is>
-          <t>1314284</t>
-        </is>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>LT02 MOLENDINAR Lighting Tower LED Metro</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>name only: as LT01</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="5" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>T0002</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="n">
-        <v>26056582</v>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="E4" s="5" t="inlineStr">
-        <is>
-          <t>1264899</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>LT03 MOLENDINAR Lighting Tower LED 76500lm Hybrid</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>name only: as LT01</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>T0002</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>26056623</v>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="E5" s="5" t="inlineStr">
-        <is>
-          <t>1188888</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>LT04 MOLENDINAR Lighting Tower LED Metro</t>
-        </is>
-      </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>name only: as LT01</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>GN20</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>26102821</v>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>1276701</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>GN20-S01-Generator 365kVA Diesel</t>
-        </is>
-      </c>
-      <c r="G6" s="4" t="n"/>
-      <c r="H6" s="4" t="n"/>
-      <c r="I6" s="4" t="inlineStr">
-        <is>
-          <t>never came to site (Andrew, 22 and 25 Oct): the docket is wrong; the branch reverses it and closes line 6</t>
-        </is>
-      </c>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>Baseplan</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>GN?</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>26121298</v>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>1316182</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>GN26 CONCERT Generator - 200kVA (Diesel)</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>name only: the concert sets sit under their own references on our record</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>GN?</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>26121310</v>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E8" s="5" t="inlineStr">
-        <is>
-          <t>1316183</t>
-        </is>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>GN27 CONCERT-Generator - 200kVA (Diesel)</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>name only: as GN26</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>LT06</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>26139060</v>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>2026-10-20</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t>1224791</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>LT05/06-Lighting Tower POD Metro</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>name only: the tower pod sits under another reference on our record</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>P05</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="n">
-        <v>26064095</v>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>1320150</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>P05 Microwave Oven</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="n"/>
-      <c r="H10" s="2" t="n"/>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>not on our record</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>P05</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>26064095</v>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>1127574</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>P05 Auto Boil</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="n"/>
-      <c r="H11" s="4" t="n"/>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>our record calls it Aircon; the docket says boiler</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>CP1</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="n">
-        <v>26064099</v>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>1116687</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>CP1 Refrigerator - Large</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="n"/>
-      <c r="H12" s="2" t="n"/>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>not on our record</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>CP1</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="n">
-        <v>26064099</v>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>119810</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>CP1 Urn</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>not on our record</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>P33</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>26064103</v>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="inlineStr">
-        <is>
-          <t>1328952</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>P33 Refrigerator - Large</t>
-        </is>
-      </c>
-      <c r="G14" s="4" t="n"/>
-      <c r="H14" s="4" t="n"/>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>keying slip: our record has 1238952 on P33</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>P09</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="n">
-        <v>26076665</v>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>1254390</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>P09 Auto Boil</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="n"/>
-      <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>not on our record</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>HRP</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>26085104</v>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-17</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t>1189410</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>P36 Portable Building Shell 6.0M x 3.0M - Cyclonic Rated</t>
-        </is>
-      </c>
-      <c r="G16" s="5" t="n"/>
-      <c r="H16" s="5" t="n"/>
-      <c r="I16" s="5" t="inlineStr">
-        <is>
-          <t>name only: our record has this shell as HRP (22 Oct review: line 93 is HRP, not P36)</t>
-        </is>
-      </c>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K16" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>P58</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n">
-        <v>26088630</v>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="E17" s="5" t="inlineStr">
-        <is>
-          <t>1273656</t>
-        </is>
-      </c>
-      <c r="F17" s="5" t="inlineStr">
-        <is>
-          <t>P44 Portable Building Shell 6.0M x 3.0M - Cyclonic Rated</t>
-        </is>
-      </c>
-      <c r="G17" s="5" t="n"/>
-      <c r="H17" s="5" t="n"/>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>name only: our record has this shell as P58 (22 Oct review: line 59 is P58, not P44)</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>P39</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>26094129</v>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>1272737</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>P38 Refrigerator - Large</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="n"/>
-      <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="inlineStr">
-        <is>
-          <t>on our record under another reference</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>P38</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>26094136</v>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>1272755</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>P39 Refrigerator - Large</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="inlineStr">
-        <is>
-          <t>on our record under another reference</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K19" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>P66</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="n">
-        <v>26126001</v>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>1311990</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>P66 Refrigerator - Large</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="n"/>
-      <c r="H20" s="4" t="n"/>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>keying slip: our record has 131190 on P66</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>P51</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>26126190</v>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>1328959</t>
-        </is>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>P46 Refrigerator - Large</t>
-        </is>
-      </c>
-      <c r="G21" s="2" t="n"/>
-      <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>on our record under another reference</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K21" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>P46, P54</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>26126190</v>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-12</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>1328957</t>
-        </is>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>P51 Refrigerator - Large</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="n"/>
-      <c r="H22" s="2" t="n"/>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>on our record under another reference</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>WC21</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>26064136</v>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>1083399</t>
-        </is>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>WC21 Toilet Portable - Fresh Water Flush</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="n"/>
-      <c r="H23" s="2" t="n"/>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>not on our record</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>WC07</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="n">
-        <v>26081411</v>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>1317643</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>WC07 Toilet Portable - Fresh Water Flush</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="n"/>
-      <c r="H24" s="4" t="n"/>
-      <c r="I24" s="4" t="inlineStr">
-        <is>
-          <t>keying slip: our record has 1317743 on WC07</t>
-        </is>
-      </c>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>WC67</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>26107560</v>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>172824</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t>WC01 Toilet Portable - Fresh Water Flush</t>
-        </is>
-      </c>
-      <c r="G25" s="5" t="n"/>
-      <c r="H25" s="5" t="n"/>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>placed at WC67 on our record; the docket names WC01 (where it was meant to go)</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Number</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr"/>
-      <c r="C26" s="2" t="n">
-        <v>26135873</v>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>1065384</t>
-        </is>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Laserplane</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="n"/>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>not on our record</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Number on two references</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>P26, P46</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="n"/>
-      <c r="D27" s="4" t="n"/>
-      <c r="E27" s="4" t="inlineStr">
-        <is>
-          <t>1311992</t>
-        </is>
-      </c>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>Fridge / Fridge Lge / Furniture</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="n"/>
-      <c r="H27" s="4" t="n"/>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>one number, two references on our record: keep the one it is on</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>Number on two references</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>P28, P46</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="n"/>
-      <c r="D28" s="4" t="n"/>
-      <c r="E28" s="4" t="inlineStr">
-        <is>
-          <t>1283996</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Fridge / Fridge Lge / Furniture</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="n"/>
-      <c r="H28" s="4" t="n"/>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>one number, two references on our record: keep the one it is on</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Number on two references</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>FL02, T0004</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="n"/>
-      <c r="D29" s="4" t="n"/>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>1197839</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Access &amp; plant / Forklift 2.5T / Other</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="n"/>
-      <c r="H29" s="4" t="n"/>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>one number, two references on our record: keep the one it is on</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>Number on two references</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>T0001, T0103</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="n"/>
-      <c r="D30" s="4" t="n"/>
-      <c r="E30" s="4" t="inlineStr">
-        <is>
-          <t>1211404</t>
-        </is>
-      </c>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>VMS / vms5</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="n"/>
-      <c r="H30" s="4" t="n"/>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>one number, two references on our record: keep the one it is on</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Number on two references</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>P41, P62</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="n"/>
-      <c r="D31" s="4" t="n"/>
-      <c r="E31" s="4" t="inlineStr">
-        <is>
-          <t>1189908</t>
-        </is>
-      </c>
-      <c r="F31" s="4" t="inlineStr">
-        <is>
-          <t>Air conditioner</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="n"/>
-      <c r="H31" s="4" t="n"/>
-      <c r="I31" s="4" t="inlineStr">
-        <is>
-          <t>one number, two references on our record: keep the one it is on</t>
-        </is>
-      </c>
-      <c r="J31" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K31" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
-        <is>
-          <t>Number on two references</t>
-        </is>
-      </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>P46, P54</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="n"/>
-      <c r="D32" s="4" t="n"/>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>1328957</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>Fridge</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="n"/>
-      <c r="H32" s="4" t="n"/>
-      <c r="I32" s="4" t="inlineStr">
-        <is>
-          <t>one number, two references on our record: keep the one it is on</t>
-        </is>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>T0002</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="n">
-        <v>26056582</v>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>1264899</t>
-        </is>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>Lighting towers</t>
-        </is>
-      </c>
-      <c r="G33" s="5" t="n"/>
-      <c r="H33" s="5" t="n"/>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>known: the towers went to the Molendinar council yard on 11 Sep, not to site (15 Oct review)</t>
-        </is>
-      </c>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K33" s="5" t="inlineStr">
-        <is>
-          <t>no (charged over the event)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>T0004</t>
-        </is>
-      </c>
-      <c r="C34" s="2" t="n">
-        <v>26056701</v>
-      </c>
-      <c r="D34" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="E34" s="2" t="inlineStr">
-        <is>
-          <t>1197839</t>
-        </is>
-      </c>
-      <c r="F34" s="2" t="inlineStr">
-        <is>
-          <t>Access &amp; plant</t>
-        </is>
-      </c>
-      <c r="G34" s="2" t="n"/>
-      <c r="H34" s="2" t="n"/>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>no arrival on our record</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>T0243</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="n">
-        <v>26091446</v>
-      </c>
-      <c r="D35" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="E35" s="2" t="inlineStr">
-        <is>
-          <t>1311144</t>
-        </is>
-      </c>
-      <c r="F35" s="2" t="inlineStr">
-        <is>
-          <t>Toilets &amp; amenities</t>
-        </is>
-      </c>
-      <c r="G35" s="2" t="n"/>
-      <c r="H35" s="2" t="n"/>
-      <c r="I35" s="2" t="inlineStr">
-        <is>
-          <t>no arrival on our record</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>no (charged over the event)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>FL02</t>
-        </is>
-      </c>
-      <c r="C36" s="2" t="n">
-        <v>26056701</v>
-      </c>
-      <c r="D36" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-11</t>
-        </is>
-      </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>1197839</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="G36" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-25</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="n">
-        <v>14</v>
-      </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>docket 14 day(s) before ours</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>EQ0005</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>26122181</v>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-13</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
-        <is>
-          <t>1262224</t>
-        </is>
-      </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Access &amp; plant</t>
-        </is>
-      </c>
-      <c r="G37" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-23</t>
-        </is>
-      </c>
-      <c r="H37" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>docket 10 day(s) before ours</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K37" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>WC06</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="n">
-        <v>26064136</v>
-      </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-15</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>1195658</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>Toilets &amp; amenities</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="I38" s="4" t="inlineStr">
-        <is>
-          <t>docket 8 day(s) before ours</t>
-        </is>
-      </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K38" s="4" t="inlineStr">
-        <is>
-          <t>no (charged over the event)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>EQ0001</t>
-        </is>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>26133817</v>
-      </c>
-      <c r="D39" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="E39" s="2" t="inlineStr">
-        <is>
-          <t>1220903</t>
-        </is>
-      </c>
-      <c r="F39" s="2" t="inlineStr">
-        <is>
-          <t>Access &amp; plant</t>
-        </is>
-      </c>
-      <c r="G39" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="H39" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>docket 3 day(s) before ours</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="5" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B40" s="5" t="inlineStr">
-        <is>
-          <t>T0024</t>
-        </is>
-      </c>
-      <c r="C40" s="5" t="n">
-        <v>26064235</v>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="E40" s="5" t="inlineStr">
-        <is>
-          <t>1211968</t>
-        </is>
-      </c>
-      <c r="F40" s="5" t="inlineStr">
-        <is>
-          <t>Toilets &amp; amenities</t>
-        </is>
-      </c>
-      <c r="G40" s="5" t="inlineStr">
-        <is>
-          <t>2026-09-26</t>
-        </is>
-      </c>
-      <c r="H40" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>a team reference on its own hire schedule (held out of every charge)</t>
-        </is>
-      </c>
-      <c r="J40" s="5" t="inlineStr">
-        <is>
-          <t>nobody</t>
-        </is>
-      </c>
-      <c r="K40" s="5" t="inlineStr">
-        <is>
-          <t>no (charged over the event)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>EQ0002</t>
-        </is>
-      </c>
-      <c r="C41" s="2" t="n">
-        <v>26141428</v>
-      </c>
-      <c r="D41" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E41" s="2" t="inlineStr">
-        <is>
-          <t>1300290</t>
-        </is>
-      </c>
-      <c r="F41" s="2" t="inlineStr">
-        <is>
-          <t>Access &amp; plant</t>
-        </is>
-      </c>
-      <c r="G41" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>docket 1 day(s) before ours</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>EQ0003</t>
-        </is>
-      </c>
-      <c r="C42" s="2" t="n">
-        <v>26141448</v>
-      </c>
-      <c r="D42" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-21</t>
-        </is>
-      </c>
-      <c r="E42" s="2" t="inlineStr">
-        <is>
-          <t>1286482</t>
-        </is>
-      </c>
-      <c r="F42" s="2" t="inlineStr">
-        <is>
-          <t>Access &amp; plant</t>
-        </is>
-      </c>
-      <c r="G42" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-22</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>docket 1 day(s) before ours</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="4" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B43" s="4" t="inlineStr">
-        <is>
-          <t>P44</t>
-        </is>
-      </c>
-      <c r="C43" s="4" t="n">
-        <v>26088639</v>
-      </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>198481</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>Portable buildings</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-24</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I43" s="4" t="inlineStr">
-        <is>
-          <t>docket 1 day(s) before ours</t>
-        </is>
-      </c>
-      <c r="J43" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K43" s="4" t="inlineStr">
-        <is>
-          <t>no (charged over the event)</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="4" t="inlineStr">
-        <is>
-          <t>Arrival</t>
-        </is>
-      </c>
-      <c r="B44" s="4" t="inlineStr">
-        <is>
-          <t>WC67</t>
-        </is>
-      </c>
-      <c r="C44" s="4" t="n">
-        <v>26107560</v>
-      </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>172824</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>Toilets &amp; amenities</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr">
-        <is>
-          <t>2026-10-01</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I44" s="4" t="inlineStr">
-        <is>
-          <t>docket 1 day(s) before ours</t>
-        </is>
-      </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>Our record</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="inlineStr">
-        <is>
-          <t>no (charged over the event)</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Barrier arrival</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>no barrier reference went in that day</t>
-        </is>
-      </c>
-      <c r="C45" s="2" t="n">
-        <v>26079322</v>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-18</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>ARMORZONMASHTL2</t>
-        </is>
-      </c>
-      <c r="F45" s="2" t="inlineStr">
-        <is>
-          <t>WB03 Barrier - Crash Rated Water filled - Armorzone MASH TL2</t>
-        </is>
-      </c>
-      <c r="G45" s="2" t="n"/>
-      <c r="H45" s="2" t="n"/>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>a barrier docket with no matching day on our record (WB03 went in 23 Sep on ours; Baseplan has 18 Sep)</t>
-        </is>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>VMS arrival</t>
-        </is>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>VMS09</t>
-        </is>
-      </c>
-      <c r="C46" s="2" t="n"/>
-      <c r="D46" s="2" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="E46" s="2" t="inlineStr">
-        <is>
-          <t>1211404</t>
-        </is>
-      </c>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t>Variable message board</t>
-        </is>
-      </c>
-      <c r="G46" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="I46" s="2" t="inlineStr">
-        <is>
-          <t>docket out 2026-09-07, 2026-10-12; in 2026-10-12</t>
-        </is>
-      </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K46" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>VMS arrival</t>
-        </is>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>VMS13</t>
-        </is>
-      </c>
-      <c r="C47" s="2" t="n"/>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-16</t>
-        </is>
-      </c>
-      <c r="E47" s="2" t="inlineStr">
-        <is>
-          <t>1191957</t>
-        </is>
-      </c>
-      <c r="F47" s="2" t="inlineStr">
-        <is>
-          <t>Variable message board</t>
-        </is>
-      </c>
-      <c r="G47" s="2" t="inlineStr">
-        <is>
-          <t>2026-10-19</t>
-        </is>
-      </c>
-      <c r="H47" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="I47" s="2" t="inlineStr">
-        <is>
-          <t>docket out 2026-10-16</t>
-        </is>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>Andrew</t>
-        </is>
-      </c>
-      <c r="K47" s="2" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -45078,4 +42613,160 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Asset no</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Turned up</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>P&amp;L branch</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="6" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="inlineStr">
+        <is>
+          <t>Building 6m</t>
+        </is>
+      </c>
+      <c r="C2" s="6" t="inlineStr">
+        <is>
+          <t>142514</t>
+        </is>
+      </c>
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>KINP</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>HRP</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>Building 6m</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>1189410</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>KINP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>FR01</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>Fridge</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>1129733</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>KINP</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>FR02</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Fridge</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>1157786</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>KINP</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
GN20 is on site: keep its Baseplan line and count its legs
Andrew corrected his earlier word: the 365 kVA set 1276701 (GN20) is
on site. The review keeps 9961976 line 6 and its labour line 52, and
asks for 4 large-set transport legs on line 55 instead of 2. Our
record and the P&L still need GN20 put back; that waits on his word.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Baseplan7_vs_Site_25Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_25Oct2026_baseplan7/GC500_Baseplan7_vs_Site_25Oct2026.xlsx
@@ -2648,7 +2648,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>55</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -2658,21 +2658,21 @@
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Labour Charge: 2 x $333.12</t>
+          <t>Transport Charge: 2 x $600.00</t>
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>1 on site (GN23); the second was GN20, which never came to site (Andrew, 22 and 25 Oct)</t>
+          <t>4 on site (GN20, GN23 x 2 legs)</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
         <is>
-          <t>Quantity 1</t>
+          <t>Quantity 4</t>
         </is>
       </c>
       <c r="G56" s="3" t="n">
-        <v>-333.12</v>
+        <v>1200</v>
       </c>
       <c r="H56" s="3" t="inlineStr">
         <is>
@@ -3193,12 +3193,12 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>9961976</t>
+          <t>9968955</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>154</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -3208,21 +3208,21 @@
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>GN20-S01-Generator 365kVA Diesel (1276701) Delivered at $6,260.40</t>
+          <t>PG29 Toilet FWF at $90.07</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
         <is>
-          <t>GN20's 365 kVA never came to site (Andrew, 22 Oct 2026, and again 25 Oct: "this never came to site 1276701 Generator 365kVA Diesel"). Coates' docket 26102821 (out 30 Sep) and the line's Delivered status are wrong: the branch reverses the docket</t>
+          <t>PG29 is on its own hire schedule (held out of every charge, Andrew 23 Oct)</t>
         </is>
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>Reverse docket 26102821 and close the line (no charge)</t>
+          <t>Take the line off this contract</t>
         </is>
       </c>
       <c r="G70" s="3" t="n">
-        <v>-6260.4</v>
+        <v>-90.06999999999999</v>
       </c>
       <c r="H70" s="3" t="inlineStr">
         <is>
@@ -3231,80 +3231,78 @@
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="3" t="inlineStr">
+      <c r="A71" s="5" t="inlineStr">
         <is>
           <t>9968955</t>
         </is>
       </c>
-      <c r="B71" s="3" t="inlineStr">
-        <is>
-          <t>154</t>
-        </is>
-      </c>
-      <c r="C71" s="3" t="inlineStr">
-        <is>
-          <t>Remove</t>
-        </is>
-      </c>
-      <c r="D71" s="3" t="inlineStr">
-        <is>
-          <t>PG29 Toilet FWF at $90.07</t>
-        </is>
-      </c>
-      <c r="E71" s="3" t="inlineStr">
-        <is>
-          <t>PG29 is on its own hire schedule (held out of every charge, Andrew 23 Oct)</t>
-        </is>
-      </c>
-      <c r="F71" s="3" t="inlineStr">
-        <is>
-          <t>Take the line off this contract</t>
-        </is>
-      </c>
-      <c r="G71" s="3" t="n">
-        <v>-90.06999999999999</v>
-      </c>
-      <c r="H71" s="3" t="inlineStr">
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>38</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>Asset number</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>WC07 asset 1317643</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>WC07 on site carries 1002538, 1002566, 1002651, 1002715, 1083300, 1181004, 1192643, 1200595, 1211959, 1212552, 1317626, 1317632, 1317640, 1317641, 1317647, 1317648, 1317649, 1317652, 1317658, 1317743</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>Correct the number on the line (the site number stands)</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="n"/>
+      <c r="H71" s="5" t="inlineStr">
         <is>
           <t>Baseplan</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>9968955</t>
-        </is>
-      </c>
-      <c r="B72" s="5" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>Asset number</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>WC07 asset 1317643</t>
-        </is>
-      </c>
-      <c r="E72" s="5" t="inlineStr">
-        <is>
-          <t>WC07 on site carries 1002538, 1002566, 1002651, 1002715, 1083300, 1181004, 1192643, 1200595, 1211959, 1212552, 1317626, 1317632, 1317640, 1317641, 1317647, 1317648, 1317649, 1317652, 1317658, 1317743</t>
-        </is>
-      </c>
-      <c r="F72" s="5" t="inlineStr">
-        <is>
-          <t>Correct the number on the line (the site number stands)</t>
-        </is>
-      </c>
-      <c r="G72" s="5" t="n"/>
-      <c r="H72" s="5" t="inlineStr">
-        <is>
-          <t>Baseplan</t>
+      <c r="A72" s="4" t="inlineStr">
+        <is>
+          <t>our record</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>GN20</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>Not on site</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>GN20 365 kVA (1276701) is Delivered from Wed 30 Sep on Baseplan, as it should be</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="inlineStr">
+        <is>
+          <t>our record deleted GN20 on 20 Oct and the P&amp;L stopped charging it on 22 Oct (v11.18)</t>
+        </is>
+      </c>
+      <c r="F72" s="4" t="inlineStr">
+        <is>
+          <t>Put it back on our record and the P&amp;L (the page will not re-use a deleted reference)</t>
+        </is>
+      </c>
+      <c r="G72" s="4" t="n"/>
+      <c r="H72" s="4" t="inlineStr">
+        <is>
+          <t>Our record</t>
         </is>
       </c>
     </row>
@@ -3943,14 +3941,14 @@
         <v>85964.00999999999</v>
       </c>
       <c r="D3" s="6" t="n">
-        <v>-3175.12</v>
+        <v>4618.4</v>
       </c>
       <c r="E3" s="6" t="n">
         <v>28671.82</v>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>Baseplan · Hours: $15.01; Baseplan · Quantity: $-333.12; Baseplan · Rate: $3,403.39; Baseplan · Remove: $-6,260.40; Decision · Rate: $28,671.82</t>
+          <t>Baseplan · Hours: $15.01; Baseplan · Quantity: $1,200.00; Baseplan · Rate: $3,403.39; Decision · Rate: $28,671.82</t>
         </is>
       </c>
     </row>
@@ -4011,7 +4009,7 @@
         <v>1022962.43</v>
       </c>
       <c r="D6" s="6" t="n">
-        <v>127387.19</v>
+        <v>135180.71</v>
       </c>
       <c r="E6" s="6" t="n">
         <v>20073.42</v>
@@ -28341,11 +28339,19 @@
         </is>
       </c>
       <c r="L241" s="2" t="n"/>
-      <c r="M241" s="2" t="n"/>
-      <c r="N241" s="2" t="n"/>
+      <c r="M241" s="2" t="inlineStr">
+        <is>
+          <t>GN20</t>
+        </is>
+      </c>
+      <c r="N241" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
       <c r="O241" s="2" t="inlineStr">
         <is>
-          <t>GN20's 365 kVA never came to site (Andrew, 22 Oct 2026, and again 25 Oct: "this never came to site 1276701 Generator 365kVA Diesel"). Coates' docket 26102821 (out 30 Sep) and the line's Delivered status are wrong: the branch reverses the docket</t>
+          <t>GN20 on site from Wed 30 Sep (Andrew, 25 Oct: "the gn20 is here"); the line stands. Our record deleted the reference on 20 Oct and the P&amp;L dropped it on 22 Oct: both to be put back</t>
         </is>
       </c>
     </row>
@@ -40798,52 +40804,52 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>9961976</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
         <is>
           <t>52</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Labour Charge</t>
         </is>
       </c>
-      <c r="D26" s="2" t="n">
+      <c r="D26" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="5" t="n">
         <v>333.12</v>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="F26" s="5" t="n">
         <v>666.24</v>
       </c>
-      <c r="G26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>333.12</v>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>1 large set on site: GN23 (GN20 never came to site; Andrew, 22 and 25 Oct)</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>Baseplan 2, ours 1</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="G26" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>666.24</v>
+      </c>
+      <c r="I26" s="5" t="inlineStr">
+        <is>
+          <t>2 large sets on site: GN20, GN23</t>
+        </is>
+      </c>
+      <c r="J26" s="5" t="inlineStr">
+        <is>
+          <t>agrees</t>
+        </is>
+      </c>
+      <c r="K26" s="5" t="inlineStr">
         <is>
           <t>NVAC-INS</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L26" s="5" t="inlineStr">
         <is>
           <t>NVAC</t>
         </is>
@@ -40954,52 +40960,52 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>9961976</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>55</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Transport Charge</t>
         </is>
       </c>
-      <c r="D29" s="5" t="n">
+      <c r="D29" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="E29" s="5" t="n">
+      <c r="E29" s="2" t="n">
         <v>600</v>
       </c>
-      <c r="F29" s="5" t="n">
+      <c r="F29" s="2" t="n">
         <v>1200</v>
       </c>
-      <c r="G29" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="H29" s="5" t="n">
-        <v>1200</v>
-      </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>1 large set x 2 legs</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>agrees</t>
-        </is>
-      </c>
-      <c r="K29" s="5" t="inlineStr">
+      <c r="G29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>2400</v>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>2 large sets (GN20, GN23) x 2 legs</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Baseplan 2, ours 4</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>NVAC-FRI</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>NVAC</t>
         </is>
@@ -41874,10 +41880,14 @@
           <t>1276701</t>
         </is>
       </c>
-      <c r="E2" s="6" t="n"/>
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>GN20</t>
+        </is>
+      </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="G2" s="6" t="inlineStr">
@@ -41889,7 +41899,11 @@
         <v>6260.4</v>
       </c>
       <c r="I2" s="6" t="n"/>
-      <c r="J2" s="6" t="n"/>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
+          <t>off the P&amp;L since 22 Oct: to be put back</t>
+        </is>
+      </c>
       <c r="K2" s="6" t="inlineStr">
         <is>
           <t>NVAC-HIR</t>

</xml_diff>